<commit_message>
docs: update literature review and project plan
- Add 11 papers (LongVidSearch, EduVidQA, Vgent, NA-VQA, 7 Video RAG)
- Rewrite Section 8 with EduVidQA/NA-VQA/LongVidSearch triangulation
- Add 4-column comparison table + dimension glossary in Section 8
- Add Gap column to Section 9 comparison table
- Merge duplicate clusters in Paper Clusters.xlsx
- Fix factual errors: redundant citation, Whisper-AT/Flamingo miscategorized
- Remove Stanford videos from PROJECT_PLAN.md; fix lecture IDs

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/literature-review/Paper Clusters.xlsx
+++ b/literature-review/Paper Clusters.xlsx
@@ -62,7 +62,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -76,11 +76,39 @@
       <top style="thin"/>
       <bottom style="thin"/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -94,6 +122,8 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -459,7 +489,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="51" customWidth="1" min="1" max="1"/>
@@ -473,6 +503,8 @@
           <t>Long-Lecture Video RAG Benchmark</t>
         </is>
       </c>
+      <c r="B1" s="5" t="n"/>
+      <c r="C1" s="6" t="n"/>
     </row>
     <row r="2" ht="6" customHeight="1"/>
     <row r="3" ht="22" customHeight="1">
@@ -504,7 +536,7 @@
         </is>
       </c>
       <c r="C4" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
@@ -579,9 +611,26 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>3</v>
-      </c>
-    </row>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Video RAG Systems</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Retrieval-Augmented Generation frameworks designed specifically for video content, including corpus-level video retrieval, long-video comprehension with RAG, and multimodal retrieval pipelines that combine transcript and visual signals.</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1"/>
+    <row r="12" ht="18" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:C1"/>

</xml_diff>